<commit_message>
Added a new row to the Excel file
</commit_message>
<xml_diff>
--- a/Price Data.xlsx
+++ b/Price Data.xlsx
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N447"/>
+  <dimension ref="A1:N448"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -13334,6 +13334,52 @@
         <v>0.1490024287395885</v>
       </c>
     </row>
+    <row r="448">
+      <c r="A448" t="inlineStr">
+        <is>
+          <t>2026-09-06 00:00:00</t>
+        </is>
+      </c>
+      <c r="B448" t="n">
+        <v>152000</v>
+      </c>
+      <c r="C448" t="n">
+        <v>22564.99</v>
+      </c>
+      <c r="D448" t="n">
+        <v>19969.01</v>
+      </c>
+      <c r="E448" t="n">
+        <v>109975</v>
+      </c>
+      <c r="F448" t="n">
+        <v>16326.21</v>
+      </c>
+      <c r="G448" t="n">
+        <v>14447.98</v>
+      </c>
+      <c r="H448" t="n">
+        <v>24360</v>
+      </c>
+      <c r="I448" t="n">
+        <v>3616.34</v>
+      </c>
+      <c r="J448" t="n">
+        <v>3200.3</v>
+      </c>
+      <c r="K448" t="n">
+        <v>120000</v>
+      </c>
+      <c r="L448" t="n">
+        <v>17814.46</v>
+      </c>
+      <c r="M448" t="n">
+        <v>15765.01</v>
+      </c>
+      <c r="N448" t="n">
+        <v>0.1490024287395885</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>